<commit_message>
task: rename project fix: Namespaces in tests task: Merge benchmarks docs: Update docs
</commit_message>
<xml_diff>
--- a/XLibur.Tests/Resource/Examples/PageSetup/HeaderFooters.xlsx
+++ b/XLibur.Tests/Resource/Examples/PageSetup/HeaderFooters.xlsx
@@ -370,11 +370,11 @@
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
   <x:headerFooter differentOddEven="0" differentFirst="0" scaleWithDoc="0" alignWithMargins="0">
-    <x:oddHeader>&amp;LCreated with XLibur</x:oddHeader>
+    <x:oddHeader>&amp;LCreated with ClosedXML</x:oddHeader>
     <x:oddFooter>&amp;C&amp;P / &amp;N&amp;R&amp;Z&amp;F</x:oddFooter>
-    <x:evenHeader>&amp;LCreated with XLibur</x:evenHeader>
+    <x:evenHeader>&amp;LCreated with ClosedXML</x:evenHeader>
     <x:evenFooter>&amp;C&amp;P / &amp;N</x:evenFooter>
-    <x:firstHeader>&amp;LCreated with XLibur&amp;R&amp;"-,Bold"The &amp;"-,Regular"&amp;KFF0000First &amp;"-,Regular"&amp;E&amp;K0000FFColorful &amp;E&amp;"Broadway,Bold Italic"&amp;K000000Page</x:firstHeader>
+    <x:firstHeader>&amp;LCreated with ClosedXML&amp;R&amp;"-,Bold"The &amp;"-,Regular"&amp;KFF0000First &amp;"-,Regular"&amp;E&amp;K0000FFColorful &amp;E&amp;"Broadway,Bold Italic"&amp;K000000Page</x:firstHeader>
     <x:firstFooter>&amp;C&amp;P / &amp;N</x:firstFooter>
   </x:headerFooter>
   <x:tableParts count="0"/>

</xml_diff>

<commit_message>
fix: update HeaderFooters reference file and improve XML attribute comparison
Update stale reference xlsx and sort XML attributes by full qualified name
(namespace + local name) for deterministic comparison across runtimes.

Co-Authored-By: @luigi-iss
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/XLibur.Tests/Resource/Examples/PageSetup/HeaderFooters.xlsx
+++ b/XLibur.Tests/Resource/Examples/PageSetup/HeaderFooters.xlsx
@@ -370,11 +370,11 @@
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
   <x:headerFooter differentOddEven="0" differentFirst="0" scaleWithDoc="0" alignWithMargins="0">
-    <x:oddHeader>&amp;LCreated with ClosedXML</x:oddHeader>
+    <x:oddHeader>&amp;LCreated with XLibur</x:oddHeader>
     <x:oddFooter>&amp;C&amp;P / &amp;N&amp;R&amp;Z&amp;F</x:oddFooter>
-    <x:evenHeader>&amp;LCreated with ClosedXML</x:evenHeader>
+    <x:evenHeader>&amp;LCreated with XLibur</x:evenHeader>
     <x:evenFooter>&amp;C&amp;P / &amp;N</x:evenFooter>
-    <x:firstHeader>&amp;LCreated with ClosedXML&amp;R&amp;"-,Bold"The &amp;"-,Regular"&amp;KFF0000First &amp;"-,Regular"&amp;E&amp;K0000FFColorful &amp;E&amp;"Broadway,Bold Italic"&amp;K000000Page</x:firstHeader>
+    <x:firstHeader>&amp;LCreated with XLibur&amp;R&amp;"-,Bold"The &amp;"-,Regular"&amp;KFF0000First &amp;"-,Regular"&amp;E&amp;K0000FFColorful &amp;E&amp;"Broadway,Bold Italic"&amp;K000000Page</x:firstHeader>
     <x:firstFooter>&amp;C&amp;P / &amp;N</x:firstFooter>
   </x:headerFooter>
   <x:tableParts count="0"/>

</xml_diff>

<commit_message>
fix: update HeaderFooters reference xlsx for XLibur rename
The reference file contained "Created with ClosedXML" headers but the
code now generates "Created with XLibur" after the project rename.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/XLibur.Tests/Resource/Examples/PageSetup/HeaderFooters.xlsx
+++ b/XLibur.Tests/Resource/Examples/PageSetup/HeaderFooters.xlsx
@@ -370,11 +370,11 @@
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
   <x:headerFooter differentOddEven="0" differentFirst="0" scaleWithDoc="0" alignWithMargins="0">
-    <x:oddHeader>&amp;LCreated with ClosedXML</x:oddHeader>
+    <x:oddHeader>&amp;LCreated with XLibur</x:oddHeader>
     <x:oddFooter>&amp;C&amp;P / &amp;N&amp;R&amp;Z&amp;F</x:oddFooter>
-    <x:evenHeader>&amp;LCreated with ClosedXML</x:evenHeader>
+    <x:evenHeader>&amp;LCreated with XLibur</x:evenHeader>
     <x:evenFooter>&amp;C&amp;P / &amp;N</x:evenFooter>
-    <x:firstHeader>&amp;LCreated with ClosedXML&amp;R&amp;"-,Bold"The &amp;"-,Regular"&amp;KFF0000First &amp;"-,Regular"&amp;E&amp;K0000FFColorful &amp;E&amp;"Broadway,Bold Italic"&amp;K000000Page</x:firstHeader>
+    <x:firstHeader>&amp;LCreated with XLibur&amp;R&amp;"-,Bold"The &amp;"-,Regular"&amp;KFF0000First &amp;"-,Regular"&amp;E&amp;K0000FFColorful &amp;E&amp;"Broadway,Bold Italic"&amp;K000000Page</x:firstHeader>
     <x:firstFooter>&amp;C&amp;P / &amp;N</x:firstFooter>
   </x:headerFooter>
   <x:tableParts count="0"/>

</xml_diff>